<commit_message>
Walk a provider ladder for recovery notices, and carry vendor email
Meta's WhatsApp Cloud API first (free tier, and template-based because Indian
recipients only accept business-initiated templates), then email — SendGrid or
any SMTP server — then Twilio, and only then a clearly labelled audited
simulation. Phones are normalised before the branch and every attempt is
audited, so a simulated send can never pass as delivered. The register gains
vendor_email per vendor, which gives the zero-cost email channel somewhere to
go, and the fixture oracle and its checks know the new column.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample_purchase_register.xlsx
+++ b/fixtures/sample_purchase_register.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,11 @@
           <t>vendor_phone</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>vendor_email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,6 +534,11 @@
           <t>+919822011456</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>accounts@sunrisepolymers.in</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -574,6 +584,11 @@
           <t>+919845023347</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>accounts@bharatofficesupplies.in</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -619,6 +634,11 @@
           <t>+919701133254</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>accounts@deccanchemicals.in</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -664,6 +684,11 @@
           <t>+919886244510</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>accounts@kaveripackaging.in</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -709,6 +734,11 @@
           <t>+919920355628</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>accounts@tridentfacilities.in</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -754,6 +784,11 @@
           <t>+919833366741</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>accounts@orionelectronics.in</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -799,6 +834,11 @@
           <t>+919876543210</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>accounts@acmecorp.in</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -844,6 +884,11 @@
           <t>+919930588774</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>accounts@zenithlogistics.in</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -889,6 +934,11 @@
           <t>+919702599806</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>accounts@nimbuscloud.in</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -934,6 +984,11 @@
           <t>+919820177890</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>accounts@vertexindustrial.in</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -979,6 +1034,11 @@
           <t>+919845288925</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>accounts@marathonfreight.in</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1022,6 +1082,11 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>+919762399462</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>accounts@sahyadrihardware.in</t>
         </is>
       </c>
     </row>

</xml_diff>